<commit_message>
fix(prestamos): la cuota del cronograma se redondea hacia arriba
Con ROUND, 1000 en 3 cuotas daba 333.33 y dejaba 0.01 de saldo. Como el
motor descuenta MIN(cuota, saldo), ese centimo se cobraba como una cuarta
cuota, un mes despues de que el trabajador termino de pagar.

Con ROUNDUP la cuota queda en 333.34 y el prestamo cierra en las 3 cuotas
pactadas, con la ultima ajustandose al saldo (333.32). El formato impreso
y el calculo de planilla vuelven a coincidir.

Verificado con 3000/6, 1000/3, 2500/7, 850/4, 100/12 y 1234.56/5: los seis
cierran en el numero de cuotas pactado y con saldo cero.

Claude-Session: https://claude.ai/code/session_01ADLMDjESZ2n5PCcyi99NHp
</commit_message>
<xml_diff>
--- a/docs/formatos/cronograma-prestamo.xlsx
+++ b/docs/formatos/cronograma-prestamo.xlsx
@@ -1138,7 +1138,7 @@
         <v>22</v>
       </c>
       <c r="B16" s="9">
-        <f>IF(N(B15)&gt;0,ROUND(B14/B15,2),0)</f>
+        <f>IF(N(B15)&gt;0,ROUNDUP(B14/B15,2),0)</f>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -2221,7 +2221,7 @@
         <v>22</v>
       </c>
       <c r="B16" s="9">
-        <f>IF(N(B15)&gt;0,ROUND(B14/B15,2),0)</f>
+        <f>IF(N(B15)&gt;0,ROUNDUP(B14/B15,2),0)</f>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>

</xml_diff>